<commit_message>
added logs of previous testcases & add multiple testcases from csv file(updated)
</commit_message>
<xml_diff>
--- a/ideakicks-test-report.csv (2).xlsx
+++ b/ideakicks-test-report.csv (2).xlsx
@@ -478,7 +478,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G5" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H5" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -782,7 +782,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G13" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H13" t="str">
         <v>latest</v>
@@ -820,7 +820,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G14" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H14" t="str">
         <v>latest</v>
@@ -858,7 +858,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G15" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H15" t="str">
         <v>latest</v>
@@ -896,7 +896,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G16" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H16" t="str">
         <v>latest</v>
@@ -934,7 +934,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G17" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H17" t="str">
         <v>latest</v>
@@ -1010,7 +1010,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G19" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H19" t="str">
         <v>2026-09-07 13-45-56</v>
@@ -1048,7 +1048,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G20" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H20" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1086,7 +1086,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G21" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H21" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1162,7 +1162,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G23" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H23" t="str">
         <v>2026-09-07 13-35-46</v>
@@ -1200,7 +1200,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G24" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H24" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1238,7 +1238,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G25" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H25" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1276,7 +1276,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G26" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H26" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1314,7 +1314,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G27" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H27" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1694,7 +1694,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G37" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H37" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1732,7 +1732,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G38" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H38" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1770,7 +1770,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G39" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H39" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1808,7 +1808,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G40" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H40" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1846,7 +1846,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G41" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H41" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1884,7 +1884,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G42" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H42" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1922,7 +1922,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G43" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H43" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1960,7 +1960,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G44" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H44" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -1998,7 +1998,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G45" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H45" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2036,7 +2036,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G46" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H46" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2112,7 +2112,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G48" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H48" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2150,7 +2150,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G49" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H49" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2188,7 +2188,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G50" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H50" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2226,7 +2226,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G51" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H51" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2264,7 +2264,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G52" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H52" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2302,7 +2302,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G53" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H53" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2340,7 +2340,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G54" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H54" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2378,7 +2378,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G55" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H55" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -2416,7 +2416,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G56" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H56" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -3442,7 +3442,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G83" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="H83" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -3518,7 +3518,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G85" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H85" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -3594,7 +3594,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G87" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H87" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -4126,7 +4126,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G101" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H101" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -4354,7 +4354,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G107" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H107" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -4392,7 +4392,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G108" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H108" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -4506,7 +4506,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G111" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H111" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -4582,7 +4582,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G113" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H113" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -4620,7 +4620,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G114" t="str">
-        <v>SKIP</v>
+        <v>PASS</v>
       </c>
       <c r="H114" t="str">
         <v>2026-09-07 13-03-50</v>
@@ -5038,7 +5038,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G125" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H125" t="str">
         <v>-</v>
@@ -5114,7 +5114,7 @@
         <v>Playwright (Chromium)</v>
       </c>
       <c r="G127" t="str">
-        <v>AUTOMATED</v>
+        <v>PASS</v>
       </c>
       <c r="H127" t="str">
         <v>-</v>

</xml_diff>